<commit_message>
Excel 102 (extra files)
</commit_message>
<xml_diff>
--- a/excel-102/Customers-01.xlsx
+++ b/excel-102/Customers-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29826"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://officenewb-my.sharepoint.com/personal/kyle_pew_officenewb_onmicrosoft_com/Documents/MicrosoftExcelComplete-2026/Exercise Files/Excel102ExerciseFiles/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cloud\Documents\coding\excel-udemy\excel-102\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="5" documentId="8_{7EDB8433-1611-49AE-8782-70065AB22D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B56EE57-1844-44D9-A776-3E930E2476D9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{373DAD7F-F51D-49FA-B90F-F70954887242}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{373DAD7F-F51D-49FA-B90F-F70954887242}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer Info" sheetId="2" r:id="rId1"/>
@@ -2535,17 +2535,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FB0386D-50C9-4F74-A578-DE7D59AE5AA0}">
   <dimension ref="A1:H92"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="13.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="36" style="1" customWidth="1"/>
-    <col min="3" max="3" width="25.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.5546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="47" style="1" customWidth="1"/>
-    <col min="5" max="8" width="16.140625" style="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="1"/>
+    <col min="5" max="8" width="16.109375" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2571,7 +2571,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -2597,7 +2597,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
@@ -2623,7 +2623,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>23</v>
       </c>
@@ -2649,7 +2649,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>28</v>
       </c>
@@ -2675,7 +2675,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>35</v>
       </c>
@@ -2701,7 +2701,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>42</v>
       </c>
@@ -2727,7 +2727,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>48</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>55</v>
       </c>
@@ -2779,7 +2779,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>62</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>68</v>
       </c>
@@ -2831,7 +2831,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>76</v>
       </c>
@@ -2857,7 +2857,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>81</v>
       </c>
@@ -2883,7 +2883,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>88</v>
       </c>
@@ -2909,7 +2909,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>93</v>
       </c>
@@ -2935,7 +2935,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>100</v>
       </c>
@@ -2961,7 +2961,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>108</v>
       </c>
@@ -2987,7 +2987,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>113</v>
       </c>
@@ -3013,7 +3013,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>119</v>
       </c>
@@ -3039,7 +3039,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>125</v>
       </c>
@@ -3065,7 +3065,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>130</v>
       </c>
@@ -3091,7 +3091,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>137</v>
       </c>
@@ -3117,7 +3117,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>142</v>
       </c>
@@ -3143,7 +3143,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>147</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>153</v>
       </c>
@@ -3195,7 +3195,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>159</v>
       </c>
@@ -3221,7 +3221,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>165</v>
       </c>
@@ -3247,7 +3247,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>169</v>
       </c>
@@ -3273,7 +3273,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>176</v>
       </c>
@@ -3299,7 +3299,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>183</v>
       </c>
@@ -3325,7 +3325,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>189</v>
       </c>
@@ -3351,7 +3351,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>195</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>201</v>
       </c>
@@ -3403,7 +3403,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>209</v>
       </c>
@@ -3429,7 +3429,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>217</v>
       </c>
@@ -3455,7 +3455,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>224</v>
       </c>
@@ -3481,7 +3481,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>231</v>
       </c>
@@ -3507,7 +3507,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>237</v>
       </c>
@@ -3533,7 +3533,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>244</v>
       </c>
@@ -3559,7 +3559,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>251</v>
       </c>
@@ -3585,7 +3585,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>257</v>
       </c>
@@ -3611,7 +3611,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>263</v>
       </c>
@@ -3637,7 +3637,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>269</v>
       </c>
@@ -3663,7 +3663,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>275</v>
       </c>
@@ -3689,7 +3689,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>282</v>
       </c>
@@ -3715,7 +3715,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>288</v>
       </c>
@@ -3741,7 +3741,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>295</v>
       </c>
@@ -3767,7 +3767,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>302</v>
       </c>
@@ -3793,7 +3793,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>309</v>
       </c>
@@ -3819,7 +3819,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>315</v>
       </c>
@@ -3845,7 +3845,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>321</v>
       </c>
@@ -3871,7 +3871,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="52" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>328</v>
       </c>
@@ -3897,7 +3897,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>335</v>
       </c>
@@ -3923,7 +3923,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>341</v>
       </c>
@@ -3949,7 +3949,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>346</v>
       </c>
@@ -3975,7 +3975,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>350</v>
       </c>
@@ -4001,7 +4001,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>357</v>
       </c>
@@ -4027,7 +4027,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>363</v>
       </c>
@@ -4053,7 +4053,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>369</v>
       </c>
@@ -4079,7 +4079,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>374</v>
       </c>
@@ -4105,7 +4105,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>380</v>
       </c>
@@ -4131,7 +4131,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>385</v>
       </c>
@@ -4157,7 +4157,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>390</v>
       </c>
@@ -4183,7 +4183,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>395</v>
       </c>
@@ -4209,7 +4209,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>401</v>
       </c>
@@ -4235,7 +4235,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>405</v>
       </c>
@@ -4261,7 +4261,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>412</v>
       </c>
@@ -4287,7 +4287,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>418</v>
       </c>
@@ -4313,7 +4313,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>423</v>
       </c>
@@ -4339,7 +4339,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>429</v>
       </c>
@@ -4365,7 +4365,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>434</v>
       </c>
@@ -4391,7 +4391,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>441</v>
       </c>
@@ -4417,7 +4417,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>448</v>
       </c>
@@ -4443,7 +4443,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>453</v>
       </c>
@@ -4469,7 +4469,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>460</v>
       </c>
@@ -4495,7 +4495,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>465</v>
       </c>
@@ -4521,7 +4521,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>472</v>
       </c>
@@ -4547,7 +4547,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="78" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>478</v>
       </c>
@@ -4573,7 +4573,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>483</v>
       </c>
@@ -4599,7 +4599,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>490</v>
       </c>
@@ -4625,7 +4625,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>496</v>
       </c>
@@ -4651,7 +4651,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>500</v>
       </c>
@@ -4677,7 +4677,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>505</v>
       </c>
@@ -4703,7 +4703,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>511</v>
       </c>
@@ -4729,7 +4729,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="85" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>517</v>
       </c>
@@ -4755,7 +4755,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>523</v>
       </c>
@@ -4781,7 +4781,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>529</v>
       </c>
@@ -4807,7 +4807,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>535</v>
       </c>
@@ -4833,7 +4833,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>542</v>
       </c>
@@ -4859,7 +4859,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>548</v>
       </c>
@@ -4885,7 +4885,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="91" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>554</v>
       </c>
@@ -4911,7 +4911,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="15" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A92" s="3" t="s">
         <v>560</v>
       </c>

</xml_diff>